<commit_message>
underwriting agent sample: a P&L category with no mapped line reads — (not $0)
Revenue Adjustments and Expense Adjustments showed $0 on the sample's P&L although no line
was mapped to either. The engine now renders an unmapped category as absent (Portfolio Demo
f4fb435, #1495); this republishes the three affected sample files via publish_to_site.py
(scrub gate CLEAN). All other fragments and downloads are byte-identical.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-t12-analysis.xlsx
+++ b/public/downloads/underwriting-demo/sample-t12-analysis.xlsx
@@ -8090,11 +8090,11 @@
         </is>
       </c>
       <c r="B6" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A6,'T-12 Data'!$O$6:$O$135)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A6)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A6,'T-12 Data'!$O$6:$O$135),"")</f>
         <v/>
       </c>
       <c r="C6" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A6,'T-12 Data'!$P$6:$P$135)*4</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A6)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A6,'T-12 Data'!$P$6:$P$135)*4,"")</f>
         <v/>
       </c>
       <c r="D6" s="10">
@@ -8113,11 +8113,11 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A7,'T-12 Data'!$O$6:$O$135)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A7)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A7,'T-12 Data'!$O$6:$O$135),"")</f>
         <v/>
       </c>
       <c r="C7" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A7,'T-12 Data'!$P$6:$P$135)*4</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A7)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A7,'T-12 Data'!$P$6:$P$135)*4,"")</f>
         <v/>
       </c>
       <c r="D7" s="10">
@@ -8136,11 +8136,11 @@
         </is>
       </c>
       <c r="B8" s="13">
-        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A8)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A8,'T-12 Data'!$O$6:$O$135),B6+B7)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A8)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A8,'T-12 Data'!$O$6:$O$135),IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A6)+COUNTIF('T-12 Data'!$B$6:$B$135,$A7)&gt;0,IF(B6="",0,B6)+IF(B7="",0,B7),""))</f>
         <v/>
       </c>
       <c r="C8" s="13">
-        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A8)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A8,'T-12 Data'!$P$6:$P$135)*4,(C6+C7))</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A8)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A8,'T-12 Data'!$P$6:$P$135)*4,IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A6)+COUNTIF('T-12 Data'!$B$6:$B$135,$A7)&gt;0,IF(C6="",0,C6)+IF(C7="",0,C7),""))</f>
         <v/>
       </c>
       <c r="D8" s="13">
@@ -8159,11 +8159,11 @@
         </is>
       </c>
       <c r="B9" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A9,'T-12 Data'!$O$6:$O$135)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A9)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A9,'T-12 Data'!$O$6:$O$135),"")</f>
         <v/>
       </c>
       <c r="C9" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A9,'T-12 Data'!$P$6:$P$135)*4</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A9)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A9,'T-12 Data'!$P$6:$P$135)*4,"")</f>
         <v/>
       </c>
       <c r="D9" s="10">
@@ -8182,11 +8182,11 @@
         </is>
       </c>
       <c r="B10" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A10,'T-12 Data'!$O$6:$O$135)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A10)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A10,'T-12 Data'!$O$6:$O$135),"")</f>
         <v/>
       </c>
       <c r="C10" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A10,'T-12 Data'!$P$6:$P$135)*4</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A10)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A10,'T-12 Data'!$P$6:$P$135)*4,"")</f>
         <v/>
       </c>
       <c r="D10" s="10">
@@ -8205,11 +8205,11 @@
         </is>
       </c>
       <c r="B11" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A11,'T-12 Data'!$O$6:$O$135)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A11)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A11,'T-12 Data'!$O$6:$O$135),"")</f>
         <v/>
       </c>
       <c r="C11" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A11,'T-12 Data'!$P$6:$P$135)*4</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A11)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A11,'T-12 Data'!$P$6:$P$135)*4,"")</f>
         <v/>
       </c>
       <c r="D11" s="10">
@@ -8228,11 +8228,11 @@
         </is>
       </c>
       <c r="B12" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A12,'T-12 Data'!$O$6:$O$135)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A12)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A12,'T-12 Data'!$O$6:$O$135),"")</f>
         <v/>
       </c>
       <c r="C12" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A12,'T-12 Data'!$P$6:$P$135)*4</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A12)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A12,'T-12 Data'!$P$6:$P$135)*4,"")</f>
         <v/>
       </c>
       <c r="D12" s="10">
@@ -8251,11 +8251,11 @@
         </is>
       </c>
       <c r="B13" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A13,'T-12 Data'!$O$6:$O$135)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A13)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A13,'T-12 Data'!$O$6:$O$135),"")</f>
         <v/>
       </c>
       <c r="C13" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A13,'T-12 Data'!$P$6:$P$135)*4</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A13)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A13,'T-12 Data'!$P$6:$P$135)*4,"")</f>
         <v/>
       </c>
       <c r="D13" s="10">
@@ -8274,11 +8274,11 @@
         </is>
       </c>
       <c r="B14" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A14,'T-12 Data'!$O$6:$O$135)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A14)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A14,'T-12 Data'!$O$6:$O$135),"")</f>
         <v/>
       </c>
       <c r="C14" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A14,'T-12 Data'!$P$6:$P$135)*4</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A14)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A14,'T-12 Data'!$P$6:$P$135)*4,"")</f>
         <v/>
       </c>
       <c r="D14" s="10">
@@ -8297,11 +8297,11 @@
         </is>
       </c>
       <c r="B15" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A15,'T-12 Data'!$O$6:$O$135)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A15)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A15,'T-12 Data'!$O$6:$O$135),"")</f>
         <v/>
       </c>
       <c r="C15" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A15,'T-12 Data'!$P$6:$P$135)*4</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A15)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A15,'T-12 Data'!$P$6:$P$135)*4,"")</f>
         <v/>
       </c>
       <c r="D15" s="10">
@@ -8343,11 +8343,11 @@
         </is>
       </c>
       <c r="B17" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A17,'T-12 Data'!$O$6:$O$135)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A17)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A17,'T-12 Data'!$O$6:$O$135),"")</f>
         <v/>
       </c>
       <c r="C17" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A17,'T-12 Data'!$P$6:$P$135)*4</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A17)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A17,'T-12 Data'!$P$6:$P$135)*4,"")</f>
         <v/>
       </c>
       <c r="D17" s="10">
@@ -8366,11 +8366,11 @@
         </is>
       </c>
       <c r="B18" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A18,'T-12 Data'!$O$6:$O$135)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A18)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A18,'T-12 Data'!$O$6:$O$135),"")</f>
         <v/>
       </c>
       <c r="C18" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A18,'T-12 Data'!$P$6:$P$135)*4</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A18)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A18,'T-12 Data'!$P$6:$P$135)*4,"")</f>
         <v/>
       </c>
       <c r="D18" s="10">
@@ -8389,11 +8389,11 @@
         </is>
       </c>
       <c r="B19" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A19,'T-12 Data'!$O$6:$O$135)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A19)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A19,'T-12 Data'!$O$6:$O$135),"")</f>
         <v/>
       </c>
       <c r="C19" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A19,'T-12 Data'!$P$6:$P$135)*4</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A19)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A19,'T-12 Data'!$P$6:$P$135)*4,"")</f>
         <v/>
       </c>
       <c r="D19" s="10">
@@ -8412,11 +8412,11 @@
         </is>
       </c>
       <c r="B20" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A20,'T-12 Data'!$O$6:$O$135)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A20)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A20,'T-12 Data'!$O$6:$O$135),"")</f>
         <v/>
       </c>
       <c r="C20" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A20,'T-12 Data'!$P$6:$P$135)*4</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A20)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A20,'T-12 Data'!$P$6:$P$135)*4,"")</f>
         <v/>
       </c>
       <c r="D20" s="10">
@@ -8435,11 +8435,11 @@
         </is>
       </c>
       <c r="B21" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A21,'T-12 Data'!$O$6:$O$135)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A21)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A21,'T-12 Data'!$O$6:$O$135),"")</f>
         <v/>
       </c>
       <c r="C21" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A21,'T-12 Data'!$P$6:$P$135)*4</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A21)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A21,'T-12 Data'!$P$6:$P$135)*4,"")</f>
         <v/>
       </c>
       <c r="D21" s="10">
@@ -8458,11 +8458,11 @@
         </is>
       </c>
       <c r="B22" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A22,'T-12 Data'!$O$6:$O$135)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A22)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A22,'T-12 Data'!$O$6:$O$135),"")</f>
         <v/>
       </c>
       <c r="C22" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A22,'T-12 Data'!$P$6:$P$135)*4</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A22)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A22,'T-12 Data'!$P$6:$P$135)*4,"")</f>
         <v/>
       </c>
       <c r="D22" s="10">
@@ -8481,11 +8481,11 @@
         </is>
       </c>
       <c r="B23" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A23,'T-12 Data'!$O$6:$O$135)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A23)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A23,'T-12 Data'!$O$6:$O$135),"")</f>
         <v/>
       </c>
       <c r="C23" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A23,'T-12 Data'!$P$6:$P$135)*4</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A23)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A23,'T-12 Data'!$P$6:$P$135)*4,"")</f>
         <v/>
       </c>
       <c r="D23" s="10">
@@ -8504,11 +8504,11 @@
         </is>
       </c>
       <c r="B24" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A24,'T-12 Data'!$O$6:$O$135)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A24)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A24,'T-12 Data'!$O$6:$O$135),"")</f>
         <v/>
       </c>
       <c r="C24" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A24,'T-12 Data'!$P$6:$P$135)*4</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A24)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A24,'T-12 Data'!$P$6:$P$135)*4,"")</f>
         <v/>
       </c>
       <c r="D24" s="10">
@@ -8527,11 +8527,11 @@
         </is>
       </c>
       <c r="B25" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A25,'T-12 Data'!$O$6:$O$135)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A25)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A25,'T-12 Data'!$O$6:$O$135),"")</f>
         <v/>
       </c>
       <c r="C25" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A25,'T-12 Data'!$P$6:$P$135)*4</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A25)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A25,'T-12 Data'!$P$6:$P$135)*4,"")</f>
         <v/>
       </c>
       <c r="D25" s="10">
@@ -8550,11 +8550,11 @@
         </is>
       </c>
       <c r="B26" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A26,'T-12 Data'!$O$6:$O$135)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A26)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A26,'T-12 Data'!$O$6:$O$135),"")</f>
         <v/>
       </c>
       <c r="C26" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A26,'T-12 Data'!$P$6:$P$135)*4</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A26)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A26,'T-12 Data'!$P$6:$P$135)*4,"")</f>
         <v/>
       </c>
       <c r="D26" s="10">
@@ -8573,11 +8573,11 @@
         </is>
       </c>
       <c r="B27" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A27,'T-12 Data'!$O$6:$O$135)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A27)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A27,'T-12 Data'!$O$6:$O$135),"")</f>
         <v/>
       </c>
       <c r="C27" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A27,'T-12 Data'!$P$6:$P$135)*4</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A27)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A27,'T-12 Data'!$P$6:$P$135)*4,"")</f>
         <v/>
       </c>
       <c r="D27" s="10">
@@ -8596,11 +8596,11 @@
         </is>
       </c>
       <c r="B28" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A28,'T-12 Data'!$O$6:$O$135)</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A28)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A28,'T-12 Data'!$O$6:$O$135),"")</f>
         <v/>
       </c>
       <c r="C28" s="10">
-        <f>SUMIF('T-12 Data'!$B$6:$B$135,$A28,'T-12 Data'!$P$6:$P$135)*4</f>
+        <f>IF(COUNTIF('T-12 Data'!$B$6:$B$135,$A28)&gt;0,SUMIF('T-12 Data'!$B$6:$B$135,$A28,'T-12 Data'!$P$6:$P$135)*4,"")</f>
         <v/>
       </c>
       <c r="D28" s="10">
@@ -9202,7 +9202,7 @@
         <v>6166658.92</v>
       </c>
       <c r="D7" s="6">
-        <f>IFERROR(B7-C7,"")</f>
+        <f>IF(C7="","",IF(B7="",0,B7)-C7)</f>
         <v/>
       </c>
       <c r="E7" s="17">
@@ -9225,7 +9225,7 @@
         <v>2054907.91</v>
       </c>
       <c r="D8" s="6">
-        <f>IFERROR(B8-C8,"")</f>
+        <f>IF(C8="","",IF(B8="",0,B8)-C8)</f>
         <v/>
       </c>
       <c r="E8" s="17">
@@ -9248,7 +9248,7 @@
         <v>4111751.01</v>
       </c>
       <c r="D9" s="6">
-        <f>IFERROR(B9-C9,"")</f>
+        <f>IF(C9="","",IF(B9="",0,B9)-C9)</f>
         <v/>
       </c>
       <c r="E9" s="17">
@@ -9269,7 +9269,7 @@
       </c>
       <c r="C10" s="17" t="n"/>
       <c r="D10" s="6">
-        <f>IFERROR(B10-C10,"")</f>
+        <f>IF(C10="","",IF(B10="",0,B10)-C10)</f>
         <v/>
       </c>
       <c r="E10" s="17">
@@ -9294,7 +9294,7 @@
       </c>
       <c r="C11" s="17" t="n"/>
       <c r="D11" s="6">
-        <f>IFERROR(B11-C11,"")</f>
+        <f>IF(C11="","",IF(B11="",0,B11)-C11)</f>
         <v/>
       </c>
       <c r="E11" s="17">
@@ -9321,7 +9321,7 @@
         <v>337165.1</v>
       </c>
       <c r="D12" s="6">
-        <f>IFERROR(B12-C12,"")</f>
+        <f>IF(C12="","",IF(B12="",0,B12)-C12)</f>
         <v/>
       </c>
       <c r="E12" s="17">

</xml_diff>